<commit_message>
(feature) : add new template for excel
</commit_message>
<xml_diff>
--- a/public/template/excel/template.xlsx
+++ b/public/template/excel/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rizdhan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03BAFD69-05C6-4F16-90CA-A224BC08F97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEB1CE0-9C40-44F3-8ADA-201C1AB503FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{48482C42-A726-4C54-9547-D22DA1E59E76}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>MOBILE_NUM</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>POL_NUM (OPTIONAL)</t>
+  </si>
+  <si>
+    <t>Text SMS</t>
+  </si>
+  <si>
+    <t>Atas pembelian ~product di Danamon, Anda mendapatkan hadiah ~amount yang telah ditransfer ke rekening Danamon Anda ~account pada ~trxdate. Info 1500090</t>
   </si>
 </sst>
 </file>
@@ -443,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A548F4-B38E-43A0-A15B-D7579DC95730}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.453125" style="3" customWidth="1"/>
@@ -456,25 +462,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
(feature) : new template excel
</commit_message>
<xml_diff>
--- a/public/template/excel/template.xlsx
+++ b/public/template/excel/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rizdhan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEB1CE0-9C40-44F3-8ADA-201C1AB503FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD0A02-6434-4859-A73D-FB8740C0A070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{48482C42-A726-4C54-9547-D22DA1E59E76}"/>
   </bookViews>
@@ -30,9 +30,6 @@
     <t>MOBILE_NUM</t>
   </si>
   <si>
-    <t>BANK_BR_CODE (OPTIONAL)</t>
-  </si>
-  <si>
     <t>BANK_ACCOUNT</t>
   </si>
   <si>
@@ -42,16 +39,19 @@
     <t>NOMINAL</t>
   </si>
   <si>
-    <t>PRODUCT_NAME (OPTIONAL)</t>
-  </si>
-  <si>
-    <t>POL_NUM (OPTIONAL)</t>
-  </si>
-  <si>
     <t>Text SMS</t>
   </si>
   <si>
-    <t>Atas pembelian ~product di Danamon, Anda mendapatkan hadiah ~amount yang telah ditransfer ke rekening Danamon Anda ~account pada ~trxdate. Info 1500090</t>
+    <t>Atas pembelian ~product di Danamon, terdapat dana masuk ke rek Danamon Anda ~account sebesar IDR ~amount pada ~trxdate. Info 1500090</t>
+  </si>
+  <si>
+    <t>POL_NUM</t>
+  </si>
+  <si>
+    <t>BANK_BR_CODE</t>
+  </si>
+  <si>
+    <t>PRODUCT_NAME</t>
   </si>
 </sst>
 </file>
@@ -463,33 +463,33 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
(feature) : new export & import
</commit_message>
<xml_diff>
--- a/public/template/excel/template.xlsx
+++ b/public/template/excel/template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rizdhan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AVELINE FELICIA\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD0A02-6434-4859-A73D-FB8740C0A070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05DF575B-547B-41A7-86C8-20613FB9DCB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{48482C42-A726-4C54-9547-D22DA1E59E76}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{48482C42-A726-4C54-9547-D22DA1E59E76}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,6 @@
     <t>FULL_NAME</t>
   </si>
   <si>
-    <t>NOMINAL</t>
-  </si>
-  <si>
     <t>Text SMS</t>
   </si>
   <si>
@@ -52,15 +49,15 @@
   </si>
   <si>
     <t>PRODUCT_NAME</t>
+  </si>
+  <si>
+    <t>JUMLAH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -70,22 +67,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -94,8 +90,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,20 +125,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -153,9 +161,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -193,7 +201,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -299,7 +307,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -441,7 +449,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -449,48 +457,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A548F4-B38E-43A0-A15B-D7579DC95730}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.453125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21" style="3" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21" style="2" customWidth="1"/>
     <col min="3" max="3" width="18.81640625" customWidth="1"/>
-    <col min="4" max="4" width="26.7265625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="30.81640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="26.7265625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="30.81640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="27.54296875" customWidth="1"/>
     <col min="7" max="7" width="34.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>8</v>
-      </c>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B3"/>
+      <c r="C3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B4"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B5"/>
+      <c r="C5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>